<commit_message>
JT-143 feat: add new full_dataset_sample.xlsx for the config scheme v8 and add full_dataset_sample_legacy.xlsx
</commit_message>
<xml_diff>
--- a/resources/Samples/full_dataset_sample_legacy.xlsx
+++ b/resources/Samples/full_dataset_sample_legacy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E3904B-91CA-4C4A-98F0-58D7867110F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EA60565-1B81-4565-B781-3298FEEF3946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4245" yWindow="4245" windowWidth="31710" windowHeight="20325" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="4035" yWindow="2625" windowWidth="29685" windowHeight="23445" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="227">
   <si>
     <t>IssueType</t>
   </si>
@@ -528,9 +528,6 @@
   </si>
   <si>
     <t>Charts: Load Tests</t>
-  </si>
-  <si>
-    <t>Leadership</t>
   </si>
   <si>
     <t>Product</t>
@@ -1508,12 +1505,6 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <alignment vertical="top"/>
     </dxf>
     <dxf>
@@ -1661,6 +1652,12 @@
     <dxf>
       <alignment vertical="top"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1697,59 +1694,59 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AL42" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AL42" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
   <autoFilter ref="A1:AL42" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
   <tableColumns count="38">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="54"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="53"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="52"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="51"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="50">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="48">
       <calculatedColumnFormula>Config!$G$4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="49"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="48"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="47"/>
-    <tableColumn id="31" xr3:uid="{DA0D5F8E-BF5F-462C-B819-B0CE3CF6918C}" name="CF Number" dataDxfId="46"/>
-    <tableColumn id="32" xr3:uid="{49F51846-B44C-482E-BB5B-806FFDC85264}" name="CF Plain Text" dataDxfId="45"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="44"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="43"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="42"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="41"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="40">
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="47"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="45"/>
+    <tableColumn id="31" xr3:uid="{DA0D5F8E-BF5F-462C-B819-B0CE3CF6918C}" name="CF Number" dataDxfId="44"/>
+    <tableColumn id="32" xr3:uid="{49F51846-B44C-482E-BB5B-806FFDC85264}" name="CF Plain Text" dataDxfId="43"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="42"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="41"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="40"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="39"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="38">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="39"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="38"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="37"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="36"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="35"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="34"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="33"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="32"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="31"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="30"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="29"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="28"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="27"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="26"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="25">
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="37"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="36"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="35"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="34"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="33"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="32"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="31"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="30"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="29"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="28"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="27"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="26"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="25"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="24"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="23">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="24">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="22">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="23">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="21">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="22">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="20">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="21">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="19">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="20">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="18">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -1765,7 +1762,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="19">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="17">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -1775,7 +1772,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="18"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1795,8 +1792,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}" name="CfgComponents" displayName="CfgComponents" ref="I3:I11" totalsRowShown="0">
-  <autoFilter ref="I3:I11" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}" name="CfgComponents" displayName="CfgComponents" ref="I3:I13" totalsRowShown="0">
+  <autoFilter ref="I3:I13" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{10F6CCA4-1068-4FC8-AB82-E48B87DB0F71}" name="Component.Name"/>
   </tableColumns>
@@ -1828,7 +1825,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="O3:O9" totalsRowShown="0">
   <autoFilter ref="O3:O9" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1862,7 +1859,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="56"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2195,14 +2192,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F73058B-F76D-4AAE-8108-6C4469E9D8B5}">
-  <dimension ref="A1:AM42"/>
+  <dimension ref="A1:AN42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.7109375" customWidth="1"/>
     <col min="4" max="4" width="10.85546875" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.5703125" customWidth="1"/>
     <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
@@ -2221,13 +2218,13 @@
     <col min="24" max="24" width="10" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="10" customWidth="1"/>
     <col min="26" max="26" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="10" customWidth="1" outlineLevel="1"/>
-    <col min="33" max="33" width="10" customWidth="1"/>
-    <col min="34" max="34" width="8.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="35" max="36" width="13.140625" customWidth="1" outlineLevel="1"/>
-    <col min="37" max="37" width="11.42578125" customWidth="1" outlineLevel="1"/>
-    <col min="38" max="39" width="13.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="40" max="40" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="10" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="33" max="33" width="10" customWidth="1" collapsed="1"/>
+    <col min="34" max="34" width="8.7109375" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="35" max="36" width="13.140625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="37" max="37" width="11.42578125" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="38" max="39" width="13.7109375" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="40" max="40" width="36.5703125" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="42" max="42" width="18.7109375" customWidth="1"/>
     <col min="43" max="43" width="87.28515625" customWidth="1"/>
   </cols>
@@ -2261,10 +2258,10 @@
         <v>8</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>9</v>
@@ -2452,7 +2449,7 @@
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>60</v>
@@ -2460,15 +2457,13 @@
       <c r="G3" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>153</v>
-      </c>
+      <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3">
         <v>1</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>102</v>
@@ -2558,24 +2553,23 @@
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="F4" s="3" t="str">
-        <f>Config!$G$4</f>
-        <v>JITTP Version 1</v>
+        <v>160</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>104</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="3">
         <v>1</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>84</v>
@@ -2667,7 +2661,7 @@
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F5" s="3" t="str">
         <f>Config!$G$4</f>
@@ -2677,14 +2671,14 @@
         <v>105</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3">
         <v>1</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>98</v>
@@ -2776,7 +2770,7 @@
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F6" s="3" t="str">
         <f>Config!$G$4</f>
@@ -2793,7 +2787,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>103</v>
@@ -2885,7 +2879,7 @@
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F7" s="3" t="str">
         <f>Config!$G$4</f>
@@ -2902,7 +2896,7 @@
         <v>1</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L7" s="3" t="s">
         <v>116</v>
@@ -2994,7 +2988,7 @@
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F8" s="3" t="str">
         <f>Config!$G$4</f>
@@ -3011,7 +3005,7 @@
         <v>1</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>101</v>
@@ -3103,7 +3097,7 @@
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F9" s="3" t="str">
         <f>Config!$G$4</f>
@@ -3120,7 +3114,7 @@
         <v>1</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L9" s="3">
         <v>1.1000000000000001</v>
@@ -3212,7 +3206,7 @@
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F10" s="3" t="str">
         <f>Config!$G$4</f>
@@ -3229,7 +3223,7 @@
         <v>1</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>98</v>
@@ -3321,7 +3315,7 @@
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F11" s="3" t="str">
         <f>Config!$G$4</f>
@@ -3338,7 +3332,7 @@
         <v>1</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>99</v>
@@ -3430,7 +3424,7 @@
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F12" s="3" t="str">
         <f>Config!$G$4</f>
@@ -3447,7 +3441,7 @@
         <v>1</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>100</v>
@@ -3539,7 +3533,7 @@
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F13" s="3" t="str">
         <f>Config!$G$4</f>
@@ -3556,7 +3550,7 @@
         <v>1</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L13" s="3" t="s">
         <v>116</v>
@@ -3648,7 +3642,7 @@
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F14" s="3" t="str">
         <f>Config!$G$4</f>
@@ -3658,14 +3652,14 @@
         <v>104</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3">
         <v>1</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L14" s="3" t="s">
         <v>84</v>
@@ -3757,7 +3751,7 @@
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F15" s="3" t="str">
         <f>Config!$G$4</f>
@@ -3774,7 +3768,7 @@
         <v>1</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>98</v>
@@ -3866,7 +3860,7 @@
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F16" s="3" t="str">
         <f>Config!$G$4</f>
@@ -3883,7 +3877,7 @@
         <v>1</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>99</v>
@@ -3975,7 +3969,7 @@
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F17" s="3" t="str">
         <f>Config!$G$4</f>
@@ -3992,7 +3986,7 @@
         <v>1</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L17" s="3" t="s">
         <v>101</v>
@@ -4084,7 +4078,7 @@
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F18" s="3" t="str">
         <f>Config!$G$4</f>
@@ -4101,7 +4095,7 @@
         <v>1</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L18" s="3" t="s">
         <v>101</v>
@@ -4193,7 +4187,7 @@
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F19" s="3" t="str">
         <f>Config!$G$4</f>
@@ -4203,14 +4197,14 @@
         <v>104</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I19" s="3"/>
       <c r="J19" s="3">
         <v>1</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>102</v>
@@ -4300,7 +4294,7 @@
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F20" s="3" t="str">
         <f>Config!$G$4</f>
@@ -4317,7 +4311,7 @@
         <v>1</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L20" s="3" t="s">
         <v>84</v>
@@ -4409,7 +4403,7 @@
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F21" s="3" t="str">
         <f>Config!$G$4</f>
@@ -4426,7 +4420,7 @@
         <v>1</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>98</v>
@@ -4518,7 +4512,7 @@
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F22" s="3" t="str">
         <f>Config!$G$4</f>
@@ -4535,7 +4529,7 @@
         <v>1</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L22" s="3" t="s">
         <v>99</v>
@@ -4627,7 +4621,7 @@
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F23" s="3" t="str">
         <f>Config!$G$4</f>
@@ -4644,7 +4638,7 @@
         <v>1</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>116</v>
@@ -4736,7 +4730,7 @@
       </c>
       <c r="D24" s="3"/>
       <c r="E24" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F24" s="3" t="str">
         <f>Config!$G$4</f>
@@ -4753,7 +4747,7 @@
         <v>1</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L24" s="3" t="s">
         <v>101</v>
@@ -4845,7 +4839,7 @@
       </c>
       <c r="D25" s="3"/>
       <c r="E25" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F25" s="3" t="str">
         <f>Config!$G$4</f>
@@ -4862,7 +4856,7 @@
         <v>1</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>84</v>
@@ -4954,7 +4948,7 @@
       </c>
       <c r="D26" s="3"/>
       <c r="E26" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F26" s="3" t="str">
         <f>Config!$G$4</f>
@@ -4971,7 +4965,7 @@
         <v>1</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>99</v>
@@ -5063,7 +5057,7 @@
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F27" s="3" t="str">
         <f>Config!$G$4</f>
@@ -5080,7 +5074,7 @@
         <v>1</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>98</v>
@@ -5172,7 +5166,7 @@
       </c>
       <c r="D28" s="3"/>
       <c r="E28" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F28" s="3" t="str">
         <f>Config!$G$4</f>
@@ -5189,7 +5183,7 @@
         <v>1</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L28" s="3" t="s">
         <v>101</v>
@@ -5281,7 +5275,7 @@
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F29" s="3" t="str">
         <f>Config!$G$4</f>
@@ -5298,7 +5292,7 @@
         <v>1</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L29" s="3" t="s">
         <v>116</v>
@@ -5390,7 +5384,7 @@
       </c>
       <c r="D30" s="3"/>
       <c r="E30" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F30" s="3" t="str">
         <f>Config!$G$4</f>
@@ -5400,14 +5394,14 @@
         <v>105</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I30" s="3"/>
       <c r="J30" s="3">
         <v>1</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L30" s="3" t="s">
         <v>84</v>
@@ -5499,7 +5493,7 @@
       </c>
       <c r="D31" s="3"/>
       <c r="E31" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F31" s="3" t="str">
         <f>Config!$G$4</f>
@@ -5509,14 +5503,14 @@
         <v>107</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3">
         <v>1</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>98</v>
@@ -5608,7 +5602,7 @@
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F32" s="3" t="str">
         <f>Config!$G$4</f>
@@ -5625,7 +5619,7 @@
         <v>1</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L32" s="3" t="s">
         <v>99</v>
@@ -5717,7 +5711,7 @@
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F33" s="3" t="str">
         <f>Config!$G$4</f>
@@ -5734,7 +5728,7 @@
         <v>1</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L33" s="3" t="s">
         <v>101</v>
@@ -5826,7 +5820,7 @@
       </c>
       <c r="D34" s="3"/>
       <c r="E34" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F34" s="3" t="str">
         <f>Config!$G$4</f>
@@ -5843,7 +5837,7 @@
         <v>1</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L34" s="3" t="s">
         <v>101</v>
@@ -5935,7 +5929,7 @@
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F35" s="3" t="str">
         <f>Config!$G$4</f>
@@ -5952,7 +5946,7 @@
         <v>1</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L35" s="3" t="s">
         <v>84</v>
@@ -6044,7 +6038,7 @@
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F36" s="3" t="str">
         <f>Config!$G$4</f>
@@ -6061,7 +6055,7 @@
         <v>1</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L36" s="3" t="s">
         <v>98</v>
@@ -6153,7 +6147,7 @@
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F37" s="3" t="str">
         <f>Config!$G$4</f>
@@ -6170,7 +6164,7 @@
         <v>1</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L37" s="3" t="s">
         <v>99</v>
@@ -6262,7 +6256,7 @@
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F38" s="3" t="str">
         <f>Config!$G$4</f>
@@ -6279,7 +6273,7 @@
         <v>1</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L38" s="3" t="s">
         <v>101</v>
@@ -6371,7 +6365,7 @@
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F39" s="3" t="str">
         <f>Config!$G$4</f>
@@ -6388,7 +6382,7 @@
         <v>1</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L39" s="3" t="s">
         <v>101</v>
@@ -6480,7 +6474,7 @@
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F40" s="3" t="str">
         <f>Config!$G$4</f>
@@ -6497,7 +6491,7 @@
         <v>1</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L40" s="3" t="s">
         <v>84</v>
@@ -6589,7 +6583,7 @@
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F41" s="3" t="str">
         <f>Config!$G$4</f>
@@ -6606,7 +6600,7 @@
         <v>1</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L41" s="3" t="s">
         <v>98</v>
@@ -6698,7 +6692,7 @@
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F42" s="3" t="str">
         <f>Config!$G$4</f>
@@ -6715,7 +6709,7 @@
         <v>1</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L42" s="3" t="s">
         <v>101</v>
@@ -6903,6 +6897,10 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="F2:F7" calculatedColumn="1"/>
+    <ignoredError sqref="G2" listDataValidation="1"/>
+  </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>
@@ -6989,7 +6987,7 @@
       <c r="R1" s="12"/>
       <c r="S1" s="12"/>
       <c r="U1" s="12" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="V1" s="12"/>
       <c r="W1" s="12"/>
@@ -7084,13 +7082,13 @@
         <v>53</v>
       </c>
       <c r="V3" t="s">
+        <v>209</v>
+      </c>
+      <c r="W3" t="s">
         <v>210</v>
       </c>
-      <c r="W3" t="s">
+      <c r="X3" t="s">
         <v>211</v>
-      </c>
-      <c r="X3" t="s">
-        <v>212</v>
       </c>
       <c r="Z3" s="5" t="s">
         <v>64</v>
@@ -7122,17 +7120,17 @@
         <v>50</v>
       </c>
       <c r="R4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="S4" s="7"/>
       <c r="U4" t="s">
+        <v>212</v>
+      </c>
+      <c r="V4" t="s">
         <v>213</v>
       </c>
-      <c r="V4" t="s">
+      <c r="W4" t="s">
         <v>214</v>
-      </c>
-      <c r="W4" t="s">
-        <v>215</v>
       </c>
       <c r="Z4" t="str" cm="1">
         <f t="array" aca="1" ref="Z4:Z13" ca="1">_xlfn.UNIQUE((_xlfn.VSTACK(INDIRECT("CfgIssueTypes[IssueType.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]"))))</f>
@@ -7165,19 +7163,19 @@
         <v>46</v>
       </c>
       <c r="R5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="S5" s="7" t="s">
         <v>74</v>
       </c>
       <c r="U5" t="s">
+        <v>215</v>
+      </c>
+      <c r="V5" t="s">
         <v>216</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>217</v>
-      </c>
-      <c r="W5" t="s">
-        <v>218</v>
       </c>
       <c r="Z5" t="str">
         <f ca="1"/>
@@ -7195,7 +7193,7 @@
         <v>62</v>
       </c>
       <c r="I6" t="s">
-        <v>155</v>
+        <v>93</v>
       </c>
       <c r="K6" t="s">
         <v>40</v>
@@ -7207,22 +7205,22 @@
         <v>88</v>
       </c>
       <c r="Q6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="R6" s="11" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>75</v>
       </c>
       <c r="U6" t="s">
+        <v>218</v>
+      </c>
+      <c r="V6" t="s">
         <v>219</v>
       </c>
-      <c r="V6" t="s">
+      <c r="W6" t="s">
         <v>220</v>
-      </c>
-      <c r="W6" t="s">
-        <v>221</v>
       </c>
       <c r="Z6" t="str">
         <f ca="1"/>
@@ -7239,7 +7237,7 @@
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="I7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K7" t="s">
         <v>41</v>
@@ -7251,20 +7249,20 @@
         <v>42</v>
       </c>
       <c r="Q7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="R7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="S7" s="7"/>
       <c r="U7" t="s">
+        <v>221</v>
+      </c>
+      <c r="V7" t="s">
         <v>222</v>
       </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>223</v>
-      </c>
-      <c r="W7" t="s">
-        <v>224</v>
       </c>
       <c r="Z7" t="str">
         <f ca="1"/>
@@ -7281,7 +7279,7 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="I8" t="s">
-        <v>95</v>
+        <v>155</v>
       </c>
       <c r="K8" t="s">
         <v>87</v>
@@ -7290,7 +7288,7 @@
         <v>48</v>
       </c>
       <c r="Q8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
@@ -7305,19 +7303,19 @@
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="I9" t="s">
-        <v>156</v>
+        <v>97</v>
       </c>
       <c r="K9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>49</v>
       </c>
       <c r="Q9" t="s">
+        <v>202</v>
+      </c>
+      <c r="R9" t="s">
         <v>203</v>
-      </c>
-      <c r="R9" t="s">
-        <v>204</v>
       </c>
       <c r="S9" s="7"/>
       <c r="Z9" t="str">
@@ -7329,13 +7327,13 @@
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="I10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Q10" t="s">
+        <v>225</v>
+      </c>
+      <c r="R10" t="s">
         <v>226</v>
-      </c>
-      <c r="R10" t="s">
-        <v>227</v>
       </c>
       <c r="S10" s="7"/>
       <c r="Z10" t="str">
@@ -7347,7 +7345,7 @@
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="I11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="Z11" t="str">
         <f ca="1"/>
@@ -7357,6 +7355,9 @@
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
+      <c r="I12" t="s">
+        <v>156</v>
+      </c>
       <c r="Z12" t="str">
         <f ca="1"/>
         <v>Note</v>
@@ -7365,6 +7366,9 @@
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
+      <c r="I13" t="s">
+        <v>157</v>
+      </c>
       <c r="Z13" t="str">
         <f ca="1"/>
         <v>WorkItem</v>
@@ -7434,6 +7438,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -7662,27 +7686,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7699,23 +7722,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>